<commit_message>
nuevo menu y muchas cosas mas
</commit_message>
<xml_diff>
--- a/Notas/Creditos_Nymphi_Wiki_y_Final.xlsx
+++ b/Notas/Creditos_Nymphi_Wiki_y_Final.xlsx
@@ -1,30 +1,29 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Xhavi\OneDrive\Documentos\TDC\The Dex Canvas\Notas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{49CEED11-A5D5-4DC2-B7BB-3139E9DAD0CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{934BB854-5E1E-464A-9AB9-77F04096315E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2295" yWindow="2295" windowWidth="28800" windowHeight="15345" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2640" yWindow="2640" windowWidth="28800" windowHeight="15345" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
     <sheet name="Canciones" sheetId="2" r:id="rId2"/>
     <sheet name="Scripts" sheetId="5" r:id="rId3"/>
-    <sheet name="Wiki_Proyecto" sheetId="3" r:id="rId4"/>
-    <sheet name="Creditos_Finales" sheetId="4" r:id="rId5"/>
+    <sheet name="Creditos_Finales" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="348" uniqueCount="185">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="344" uniqueCount="184">
   <si>
     <t>THE DEX CANVAS</t>
   </si>
@@ -350,9 +349,6 @@
     <t>RECURSOS DE TERCEROS</t>
   </si>
   <si>
-    <t>Música</t>
-  </si>
-  <si>
     <t>Recurso</t>
   </si>
   <si>
@@ -362,22 +358,10 @@
     <t>MK_UICustomizer</t>
   </si>
   <si>
-    <t>MK_UICustomizer_Battle_lite</t>
-  </si>
-  <si>
-    <t> MOG_ActionName</t>
-  </si>
-  <si>
     <t>Aerosys</t>
   </si>
   <si>
     <t>Moghunter</t>
-  </si>
-  <si>
-    <t>Gratuita</t>
-  </si>
-  <si>
-    <t>Sprites</t>
   </si>
   <si>
     <t>AGRADECIMIENTOS ESPECIALES</t>
@@ -478,51 +462,12 @@
     <t>Moonlit lake</t>
   </si>
   <si>
-    <t>THE DEX CANVAS - WIKI DEL PROYECTO</t>
-  </si>
-  <si>
-    <t>NPCs Importantes</t>
-  </si>
-  <si>
-    <t>Nymphi</t>
-  </si>
-  <si>
     <t>Yoss</t>
   </si>
   <si>
-    <t>Dex</t>
-  </si>
-  <si>
-    <t>Mapas</t>
-  </si>
-  <si>
-    <t>Sylverain</t>
-  </si>
-  <si>
-    <t>Bosque Lumaria</t>
-  </si>
-  <si>
-    <t>Estanque Sagrado</t>
-  </si>
-  <si>
-    <t>Mecánicas</t>
-  </si>
-  <si>
-    <t>Parry</t>
-  </si>
-  <si>
-    <t>Combate</t>
-  </si>
-  <si>
-    <t>Exploración</t>
-  </si>
-  <si>
     <t>TALES OF DEX: THE NYMPHI STORY</t>
   </si>
   <si>
-    <t>Adrián González</t>
-  </si>
-  <si>
     <t>Diseño Narrativo</t>
   </si>
   <si>
@@ -577,34 +522,85 @@
     <t>Creador</t>
   </si>
   <si>
-    <t>Aura Sync</t>
-  </si>
-  <si>
-    <t>Adaptative Layout</t>
-  </si>
-  <si>
-    <t>Battle Positions</t>
-  </si>
-  <si>
-    <t>Battle Results</t>
-  </si>
-  <si>
-    <t>Map name HUD</t>
-  </si>
-  <si>
-    <t>Over Pass</t>
-  </si>
-  <si>
-    <t>Tittle Menu</t>
-  </si>
-  <si>
-    <t>MOG - Action Name</t>
-  </si>
-  <si>
     <t>Tierras de Lúmira</t>
   </si>
   <si>
     <t>The overworld</t>
+  </si>
+  <si>
+    <t>Hollow Knight</t>
+  </si>
+  <si>
+    <t>DifficultyModes</t>
+  </si>
+  <si>
+    <t>AdaptiveLayout</t>
+  </si>
+  <si>
+    <t>CreditsScene</t>
+  </si>
+  <si>
+    <t>TitleMenu</t>
+  </si>
+  <si>
+    <t>AuraSync</t>
+  </si>
+  <si>
+    <t>LimitResonance</t>
+  </si>
+  <si>
+    <t>TDC_LevelBalance</t>
+  </si>
+  <si>
+    <t>BattlerLimitGauge</t>
+  </si>
+  <si>
+    <t>Overpass.js</t>
+  </si>
+  <si>
+    <t>MapNameHud</t>
+  </si>
+  <si>
+    <t>BattlePositions</t>
+  </si>
+  <si>
+    <t>BattleResults</t>
+  </si>
+  <si>
+    <t>MK_UICustomizer_Battle_...</t>
+  </si>
+  <si>
+    <t>MOG_ActionName</t>
+  </si>
+  <si>
+    <t>EchoWhisper</t>
+  </si>
+  <si>
+    <t>EchoSense</t>
+  </si>
+  <si>
+    <t>LightingMZ</t>
+  </si>
+  <si>
+    <t>BubbleMessagesMZ</t>
+  </si>
+  <si>
+    <t>Hendrix_Event_Emitter</t>
+  </si>
+  <si>
+    <t>Sang Hendrix</t>
+  </si>
+  <si>
+    <t>Guardian Templo del viento</t>
+  </si>
+  <si>
+    <t>Tempes sentinel theme</t>
+  </si>
+  <si>
+    <t>Lunhiel</t>
+  </si>
+  <si>
+    <t>Snow over Lunhiel</t>
   </si>
 </sst>
 </file>
@@ -2265,37 +2261,29 @@
       </c>
     </row>
     <row r="359" spans="1:1" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A359" s="2" t="s">
-        <v>108</v>
-      </c>
+      <c r="A359" s="2"/>
     </row>
     <row r="360" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A360" s="3"/>
     </row>
     <row r="361" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A361" s="3" t="s">
-        <v>109</v>
-      </c>
+      <c r="A361" s="3"/>
     </row>
     <row r="362" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A362" s="3"/>
     </row>
     <row r="363" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A363" s="3" t="s">
-        <v>100</v>
-      </c>
+      <c r="A363" s="3"/>
     </row>
     <row r="364" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A364" s="3"/>
     </row>
     <row r="365" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A365" s="3" t="s">
-        <v>101</v>
-      </c>
+      <c r="A365" s="3"/>
     </row>
     <row r="367" spans="1:1" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A367" s="2" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
     </row>
     <row r="368" spans="1:1" x14ac:dyDescent="0.25">
@@ -2303,7 +2291,7 @@
     </row>
     <row r="369" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A369" s="3" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="370" spans="1:4" x14ac:dyDescent="0.25">
@@ -2323,93 +2311,54 @@
       </c>
     </row>
     <row r="375" spans="1:4" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A375" s="2" t="s">
-        <v>48</v>
-      </c>
+      <c r="A375" s="2"/>
     </row>
     <row r="376" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A376" s="3"/>
     </row>
     <row r="377" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A377" s="3" t="s">
-        <v>109</v>
-      </c>
-      <c r="B377" t="s">
-        <v>111</v>
-      </c>
-      <c r="C377" t="s">
-        <v>112</v>
-      </c>
-      <c r="D377" s="4" t="s">
-        <v>113</v>
-      </c>
+      <c r="A377" s="3"/>
+      <c r="D377" s="4"/>
     </row>
     <row r="378" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A378" s="3"/>
     </row>
     <row r="379" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A379" s="3" t="s">
-        <v>100</v>
-      </c>
-      <c r="B379" s="4" t="s">
-        <v>114</v>
-      </c>
-      <c r="C379" s="4" t="s">
-        <v>114</v>
-      </c>
-      <c r="D379" s="4" t="s">
-        <v>115</v>
-      </c>
+      <c r="A379" s="3"/>
+      <c r="B379" s="4"/>
+      <c r="C379" s="4"/>
+      <c r="D379" s="4"/>
     </row>
     <row r="380" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A380" s="3"/>
     </row>
     <row r="381" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A381" s="3" t="s">
-        <v>101</v>
-      </c>
-      <c r="B381" t="s">
-        <v>116</v>
-      </c>
-      <c r="C381" t="s">
-        <v>116</v>
-      </c>
-      <c r="D381" t="s">
-        <v>116</v>
-      </c>
+      <c r="A381" s="3"/>
     </row>
     <row r="383" spans="1:4" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A383" s="2" t="s">
-        <v>117</v>
-      </c>
+      <c r="A383" s="2"/>
     </row>
     <row r="384" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A384" s="3"/>
     </row>
     <row r="385" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A385" s="3" t="s">
-        <v>109</v>
-      </c>
+      <c r="A385" s="3"/>
     </row>
     <row r="386" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A386" s="3"/>
     </row>
     <row r="387" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A387" s="3" t="s">
-        <v>100</v>
-      </c>
+      <c r="A387" s="3"/>
     </row>
     <row r="388" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A388" s="3"/>
     </row>
     <row r="389" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A389" s="3" t="s">
-        <v>101</v>
-      </c>
+      <c r="A389" s="3"/>
     </row>
     <row r="393" spans="1:2" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A393" s="1" t="s">
-        <v>118</v>
+        <v>113</v>
       </c>
     </row>
     <row r="394" spans="1:2" x14ac:dyDescent="0.25">
@@ -2417,7 +2366,7 @@
     </row>
     <row r="395" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A395" s="3" t="s">
-        <v>119</v>
+        <v>114</v>
       </c>
     </row>
     <row r="396" spans="1:2" x14ac:dyDescent="0.25">
@@ -2425,7 +2374,7 @@
     </row>
     <row r="397" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A397" s="3" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
     </row>
     <row r="398" spans="1:2" x14ac:dyDescent="0.25">
@@ -2436,7 +2385,7 @@
         <v>82</v>
       </c>
       <c r="B399" t="s">
-        <v>121</v>
+        <v>116</v>
       </c>
     </row>
     <row r="400" spans="1:2" x14ac:dyDescent="0.25">
@@ -2444,7 +2393,7 @@
     </row>
     <row r="401" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A401" s="3" t="s">
-        <v>122</v>
+        <v>117</v>
       </c>
     </row>
     <row r="402" spans="1:1" x14ac:dyDescent="0.25">
@@ -2452,17 +2401,17 @@
     </row>
     <row r="403" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A403" s="3" t="s">
-        <v>123</v>
+        <v>118</v>
       </c>
     </row>
     <row r="407" spans="1:1" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A407" s="1" t="s">
-        <v>124</v>
+        <v>119</v>
       </c>
     </row>
     <row r="409" spans="1:1" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A409" s="2" t="s">
-        <v>125</v>
+        <v>120</v>
       </c>
     </row>
     <row r="410" spans="1:1" x14ac:dyDescent="0.25">
@@ -2470,15 +2419,17 @@
     </row>
     <row r="411" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A411" s="3" t="s">
-        <v>126</v>
+        <v>121</v>
       </c>
     </row>
     <row r="412" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A412" s="3"/>
+      <c r="A412" s="3" t="s">
+        <v>159</v>
+      </c>
     </row>
     <row r="413" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A413" s="3" t="s">
-        <v>127</v>
+        <v>122</v>
       </c>
     </row>
     <row r="414" spans="1:1" x14ac:dyDescent="0.25">
@@ -2486,7 +2437,7 @@
     </row>
     <row r="415" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A415" s="3" t="s">
-        <v>128</v>
+        <v>123</v>
       </c>
     </row>
     <row r="416" spans="1:1" x14ac:dyDescent="0.25">
@@ -2494,12 +2445,12 @@
     </row>
     <row r="417" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A417" s="3" t="s">
-        <v>129</v>
+        <v>124</v>
       </c>
     </row>
     <row r="419" spans="1:1" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A419" s="2" t="s">
-        <v>130</v>
+        <v>125</v>
       </c>
     </row>
     <row r="420" spans="1:1" x14ac:dyDescent="0.25">
@@ -2507,7 +2458,7 @@
     </row>
     <row r="421" spans="1:1" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A421" s="5" t="s">
-        <v>131</v>
+        <v>126</v>
       </c>
     </row>
     <row r="425" spans="1:1" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2517,17 +2468,17 @@
     </row>
     <row r="427" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A427" t="s">
-        <v>132</v>
+        <v>127</v>
       </c>
     </row>
     <row r="432" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A432" t="s">
-        <v>133</v>
+        <v>128</v>
       </c>
     </row>
     <row r="433" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A433" t="s">
-        <v>134</v>
+        <v>129</v>
       </c>
     </row>
   </sheetData>
@@ -2538,7 +2489,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:M14"/>
+  <dimension ref="A1:M19"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="23.85546875" bestFit="1" customWidth="1"/>
@@ -2548,10 +2499,10 @@
   <sheetData>
     <row r="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>135</v>
+        <v>130</v>
       </c>
       <c r="B1" t="s">
-        <v>136</v>
+        <v>131</v>
       </c>
       <c r="C1" t="s">
         <v>100</v>
@@ -2559,10 +2510,10 @@
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>137</v>
+        <v>132</v>
       </c>
       <c r="B2" t="s">
-        <v>137</v>
+        <v>132</v>
       </c>
       <c r="C2" t="s">
         <v>35</v>
@@ -2570,10 +2521,10 @@
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>183</v>
+        <v>157</v>
       </c>
       <c r="B3" t="s">
-        <v>184</v>
+        <v>158</v>
       </c>
       <c r="C3" t="s">
         <v>35</v>
@@ -2581,10 +2532,10 @@
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>138</v>
+        <v>133</v>
       </c>
       <c r="B4" t="s">
-        <v>139</v>
+        <v>134</v>
       </c>
       <c r="C4" t="s">
         <v>35</v>
@@ -2592,10 +2543,10 @@
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>140</v>
+        <v>135</v>
       </c>
       <c r="B5" t="s">
-        <v>141</v>
+        <v>136</v>
       </c>
       <c r="C5" t="s">
         <v>35</v>
@@ -2603,10 +2554,10 @@
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>167</v>
+        <v>149</v>
       </c>
       <c r="B6" t="s">
-        <v>168</v>
+        <v>150</v>
       </c>
       <c r="C6" t="s">
         <v>35</v>
@@ -2614,10 +2565,10 @@
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>169</v>
+        <v>151</v>
       </c>
       <c r="B7" t="s">
-        <v>170</v>
+        <v>152</v>
       </c>
       <c r="C7" t="s">
         <v>35</v>
@@ -2625,17 +2576,42 @@
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>171</v>
+        <v>154</v>
       </c>
       <c r="B8" t="s">
-        <v>172</v>
+        <v>153</v>
       </c>
       <c r="C8" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>180</v>
+      </c>
+      <c r="B9" t="s">
+        <v>181</v>
+      </c>
+      <c r="C9" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>182</v>
+      </c>
+      <c r="B10" t="s">
+        <v>183</v>
+      </c>
+      <c r="C10" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="14" spans="1:13" x14ac:dyDescent="0.25">
       <c r="M14" s="8"/>
+    </row>
+    <row r="19" spans="7:7" x14ac:dyDescent="0.25">
+      <c r="G19" s="8"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2644,7 +2620,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{64671C36-A078-4719-8615-69694B03360C}">
-  <dimension ref="A1:B9"/>
+  <dimension ref="A1:B23"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="21.5703125" bestFit="1" customWidth="1"/>
@@ -2652,15 +2628,15 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>173</v>
+        <v>155</v>
       </c>
       <c r="B1" t="s">
-        <v>174</v>
+        <v>156</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>176</v>
+        <v>161</v>
       </c>
       <c r="B2" t="s">
         <v>35</v>
@@ -2668,7 +2644,7 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>175</v>
+        <v>162</v>
       </c>
       <c r="B3" t="s">
         <v>35</v>
@@ -2676,7 +2652,7 @@
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>177</v>
+        <v>163</v>
       </c>
       <c r="B4" t="s">
         <v>35</v>
@@ -2684,7 +2660,7 @@
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>178</v>
+        <v>160</v>
       </c>
       <c r="B5" t="s">
         <v>35</v>
@@ -2692,7 +2668,7 @@
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>179</v>
+        <v>164</v>
       </c>
       <c r="B6" t="s">
         <v>35</v>
@@ -2700,7 +2676,7 @@
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>180</v>
+        <v>165</v>
       </c>
       <c r="B7" t="s">
         <v>35</v>
@@ -2708,7 +2684,7 @@
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>181</v>
+        <v>166</v>
       </c>
       <c r="B8" t="s">
         <v>35</v>
@@ -2716,10 +2692,103 @@
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>182</v>
-      </c>
-      <c r="B9" t="s">
-        <v>115</v>
+        <v>167</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>168</v>
+      </c>
+      <c r="B10" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>169</v>
+      </c>
+      <c r="B11" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>170</v>
+      </c>
+      <c r="B12" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>171</v>
+      </c>
+      <c r="B13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>110</v>
+      </c>
+      <c r="B15" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>172</v>
+      </c>
+      <c r="B16" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>173</v>
+      </c>
+      <c r="B17" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>174</v>
+      </c>
+      <c r="B18" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>175</v>
+      </c>
+      <c r="B19" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>176</v>
+      </c>
+      <c r="B21" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>177</v>
+      </c>
+      <c r="B22" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>178</v>
+      </c>
+      <c r="B23" t="s">
+        <v>179</v>
       </c>
     </row>
   </sheetData>
@@ -2728,81 +2797,6 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:A16"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>149</v>
-      </c>
-    </row>
-    <row r="11" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="13" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="14" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
-        <v>152</v>
-      </c>
-    </row>
-    <row r="15" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
-        <v>153</v>
-      </c>
-    </row>
-    <row r="16" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
-        <v>154</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:A33"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -2814,7 +2808,7 @@
     </row>
     <row r="3" spans="1:1" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A3" s="7" t="s">
-        <v>155</v>
+        <v>138</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
@@ -2824,7 +2818,7 @@
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>156</v>
+        <v>35</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.25">
@@ -2834,72 +2828,72 @@
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>156</v>
+        <v>35</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>157</v>
+        <v>139</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>156</v>
+        <v>35</v>
       </c>
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>158</v>
+        <v>140</v>
       </c>
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>156</v>
+        <v>35</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>159</v>
+        <v>141</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>160</v>
+        <v>142</v>
       </c>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>161</v>
+        <v>143</v>
       </c>
     </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>145</v>
+        <v>137</v>
       </c>
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>162</v>
+        <v>144</v>
       </c>
     </row>
     <row r="25" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>163</v>
+        <v>145</v>
       </c>
     </row>
     <row r="27" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>164</v>
+        <v>146</v>
       </c>
     </row>
     <row r="29" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>165</v>
+        <v>147</v>
       </c>
     </row>
     <row r="31" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>166</v>
+        <v>148</v>
       </c>
     </row>
     <row r="33" spans="1:1" x14ac:dyDescent="0.25">

</xml_diff>